<commit_message>
added Verteilungen darstellen as shiny-live app
</commit_message>
<xml_diff>
--- a/Block01-Methodologie/Live-Experiment-Regression_to_the_mean.xlsx
+++ b/Block01-Methodologie/Live-Experiment-Regression_to_the_mean.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelmerk/Nextcloud/Lehre/Lehre_WS_2425/VL-Forschungsmethoden-WiSe2425/Block01-Methodologie/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelmerk/Nextcloud/Lehre/Lehre_SS_25/VL-Forschungsmethoden-SoSe25/Block01-Methodologie/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB10AC86-CDE6-644A-81DB-0428C486537D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B71AD0-BDED-2E4F-9193-F2836DC6BFE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1000" windowWidth="34560" windowHeight="21100" xr2:uid="{A0494C58-B0C1-5A42-BA17-0C7F278390D5}"/>
   </bookViews>
@@ -28,7 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -214,9 +213,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 – 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -254,7 +253,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 – 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -360,7 +359,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 – 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -502,7 +501,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -840,11 +839,11 @@
         <v/>
       </c>
       <c r="C20" s="1" t="str">
-        <f t="shared" ref="C4:C67" si="3">IF(B20="JA",A20-A19,"")</f>
+        <f t="shared" ref="C20:C67" si="3">IF(B20="JA",A20-A19,"")</f>
         <v/>
       </c>
       <c r="D20" s="1" t="str">
-        <f t="shared" ref="D4:D67" si="4">IF(B20="NEIN",A20-A19,"")</f>
+        <f t="shared" ref="D20:D67" si="4">IF(B20="NEIN",A20-A19,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>